<commit_message>
Add geschaeftsreise: Hotelrechnung Hotel Reginella Roma
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q3/2026-09-22_Rom/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q3/2026-09-22_Rom/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,8 +19,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -94,7 +94,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -105,7 +105,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -124,6 +124,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -492,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -587,7 +590,7 @@
           <t>Flugticket</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n"/>
+      <c r="D2" s="11" t="n"/>
       <c r="E2" s="5" t="n">
         <v>0</v>
       </c>
@@ -602,10 +605,10 @@
           <t>Italien</t>
         </is>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="11" t="n">
         <v>46287</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="J2" s="11" t="n">
         <v>46292</v>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -619,61 +622,91 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="n"/>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Hotelrechnung-Reginella-Roma.md</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Hotelrechnung Hotel Reginella Roma</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Hotelrechnung</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="n"/>
+      <c r="E3" s="5" t="n">
+        <v>1125</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Italien</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>46287</v>
+      </c>
+      <c r="J3" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Hotelrechnung des Hotel Reginella Roma für den Aufenthalt von Dr. Michael Weber vom 22.09.2026 bis 27.09.2026 (5 Nächte) im Deluxe Business Room inklusive Frühstück, Kurtaxe und Wäscheservice.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n"/>
-      <c r="C4" s="8" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="9">
-        <f>SUM(E2:E2)</f>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="9">
+        <f>SUM(E2:E3)</f>
         <v/>
       </c>
-      <c r="F4" s="8" t="n"/>
-      <c r="G4" s="8" t="n"/>
-      <c r="H4" s="8" t="n"/>
-      <c r="I4" s="8" t="n"/>
-      <c r="J4" s="8" t="n"/>
-      <c r="K4" s="8" t="n"/>
-      <c r="L4" s="8" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="8" t="n"/>
+      <c r="H5" s="8" t="n"/>
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="8" t="n"/>
+      <c r="K5" s="8" t="n"/>
+      <c r="L5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A6" s="3" t="n"/>
       <c r="B6" s="3" t="n"/>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="3" t="n"/>
@@ -687,18 +720,15 @@
       <c r="L6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Flugticket</t>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n"/>
-      <c r="E7" s="5">
-        <f>SUMIF(C2:C2,A7,E2:E2)</f>
-        <v/>
-      </c>
+      <c r="E7" s="6" t="n"/>
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="n"/>
@@ -707,10 +737,53 @@
       <c r="K7" s="3" t="n"/>
       <c r="L7" s="3" t="n"/>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Flugticket</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="5">
+        <f>SUMIF(C2:C3,A8,E2:E3)</f>
+        <v/>
+      </c>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Hotelrechnung</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="5">
+        <f>SUMIF(C2:C3,A9,E2:E3)</f>
+        <v/>
+      </c>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L2"/>
+  <autoFilter ref="A1:L3"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Flugrechnung Rückflug Rom - Augsburg
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q3/2026-09-22_Rom/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q3/2026-09-22_Rom/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -670,61 +670,91 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Flugrechnung-Rueckflug-Rom-Augsburg.md</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Flugrechnung Rückflug Rom - Augsburg</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Flugrechnung</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="5" t="n">
+        <v>533.5</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Italien</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>46287</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Rechnung für den Rückflug von Rom Fiumicino nach München/Augsburg inkl. Flughafengebühren und Shuttle-Transfer nach Augsburg. Teil der Geschäftsreise nach Rom.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="9">
-        <f>SUM(E2:E3)</f>
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="9">
+        <f>SUM(E2:E4)</f>
         <v/>
       </c>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="8" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="8" t="n"/>
+      <c r="H6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
+      <c r="J6" s="8" t="n"/>
+      <c r="K6" s="8" t="n"/>
+      <c r="L6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A7" s="3" t="n"/>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n"/>
@@ -738,18 +768,15 @@
       <c r="L7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Flugticket</t>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="3" t="n"/>
-      <c r="E8" s="5">
-        <f>SUMIF(C2:C3,A8,E2:E3)</f>
-        <v/>
-      </c>
+      <c r="E8" s="6" t="n"/>
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="3" t="n"/>
@@ -761,14 +788,14 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Hotelrechnung</t>
+          <t>Flugticket</t>
         </is>
       </c>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n"/>
       <c r="E9" s="5">
-        <f>SUMIF(C2:C3,A9,E2:E3)</f>
+        <f>SUMIF(C2:C4,A9,E2:E4)</f>
         <v/>
       </c>
       <c r="F9" s="3" t="n"/>
@@ -779,11 +806,54 @@
       <c r="K9" s="3" t="n"/>
       <c r="L9" s="3" t="n"/>
     </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Hotelrechnung</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="5">
+        <f>SUMIF(C2:C4,A10,E2:E4)</f>
+        <v/>
+      </c>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Flugrechnung</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="5">
+        <f>SUMIF(C2:C4,A11,E2:E4)</f>
+        <v/>
+      </c>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L3"/>
+  <autoFilter ref="A1:L4"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Bewirtungsbeleg Ristorante Ragno d'Oro Rom
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q3/2026-09-22_Rom/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q3/2026-09-22_Rom/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -718,61 +718,91 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Restaurantrechnung-Ragno-dOro.md</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Bewirtungsbeleg Ristorante Ragno d'Oro Rom</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Bewirtungsbeleg</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="5" t="n">
+        <v>265</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Italien</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="n">
+        <v>46287</v>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Bewirtungsbeleg für ein Geschäftsessen im Ristorante Ragno d'Oro in Rom zwischen Dr. Michael Weber (TechInnovate Augsburg GmbH) und Dott. Marco Rossi (Italia Systems S.p.A.) zur Abstimmung der Expansion Südosteuropa &amp; IT-Integration.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="9">
-        <f>SUM(E2:E4)</f>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="9">
+        <f>SUM(E2:E5)</f>
         <v/>
       </c>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
-      <c r="L6" s="8" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
+      <c r="J7" s="8" t="n"/>
+      <c r="K7" s="8" t="n"/>
+      <c r="L7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A8" s="3" t="n"/>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="3" t="n"/>
@@ -786,18 +816,15 @@
       <c r="L8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Flugticket</t>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n"/>
-      <c r="E9" s="5">
-        <f>SUMIF(C2:C4,A9,E2:E4)</f>
-        <v/>
-      </c>
+      <c r="E9" s="6" t="n"/>
       <c r="F9" s="3" t="n"/>
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="3" t="n"/>
@@ -809,14 +836,14 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Hotelrechnung</t>
+          <t>Flugticket</t>
         </is>
       </c>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
       <c r="E10" s="5">
-        <f>SUMIF(C2:C4,A10,E2:E4)</f>
+        <f>SUMIF(C2:C5,A10,E2:E5)</f>
         <v/>
       </c>
       <c r="F10" s="3" t="n"/>
@@ -830,14 +857,14 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Flugrechnung</t>
+          <t>Hotelrechnung</t>
         </is>
       </c>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="3" t="n"/>
       <c r="E11" s="5">
-        <f>SUMIF(C2:C4,A11,E2:E4)</f>
+        <f>SUMIF(C2:C5,A11,E2:E5)</f>
         <v/>
       </c>
       <c r="F11" s="3" t="n"/>
@@ -848,12 +875,55 @@
       <c r="K11" s="3" t="n"/>
       <c r="L11" s="3" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Flugrechnung</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="5">
+        <f>SUMIF(C2:C5,A12,E2:E5)</f>
+        <v/>
+      </c>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Bewirtungsbeleg</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="5">
+        <f>SUMIF(C2:C5,A13,E2:E5)</f>
+        <v/>
+      </c>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L4"/>
+  <autoFilter ref="A1:L5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Uber Fahrtenbeleg Rom
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q3/2026-09-22_Rom/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q3/2026-09-22_Rom/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -766,61 +766,91 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Uber-Fahrtenbeleg-Rom.md</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Uber Fahrtenbeleg Rom</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Italien</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Fahrtenbeleg für eine Uber Black Fahrt in Rom vom Hotel Reginella zum Ristorante Ragno d'Oro am 25.09.2026, abgerechnet über Visa Corporate Karte im Rahmen einer Dienstreise.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="9">
-        <f>SUM(E2:E5)</f>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="9">
+        <f>SUM(E2:E6)</f>
         <v/>
       </c>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="8" t="n"/>
+      <c r="K8" s="8" t="n"/>
+      <c r="L8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A9" s="3" t="n"/>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n"/>
@@ -834,18 +864,15 @@
       <c r="L9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Flugticket</t>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
-      <c r="E10" s="5">
-        <f>SUMIF(C2:C5,A10,E2:E5)</f>
-        <v/>
-      </c>
+      <c r="E10" s="6" t="n"/>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="n"/>
@@ -857,14 +884,14 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Hotelrechnung</t>
+          <t>Flugticket</t>
         </is>
       </c>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="3" t="n"/>
       <c r="E11" s="5">
-        <f>SUMIF(C2:C5,A11,E2:E5)</f>
+        <f>SUMIF(C2:C6,A11,E2:E6)</f>
         <v/>
       </c>
       <c r="F11" s="3" t="n"/>
@@ -878,14 +905,14 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Flugrechnung</t>
+          <t>Hotelrechnung</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
       <c r="E12" s="5">
-        <f>SUMIF(C2:C5,A12,E2:E5)</f>
+        <f>SUMIF(C2:C6,A12,E2:E6)</f>
         <v/>
       </c>
       <c r="F12" s="3" t="n"/>
@@ -899,14 +926,14 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Bewirtungsbeleg</t>
+          <t>Flugrechnung</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n"/>
       <c r="E13" s="5">
-        <f>SUMIF(C2:C5,A13,E2:E5)</f>
+        <f>SUMIF(C2:C6,A13,E2:E6)</f>
         <v/>
       </c>
       <c r="F13" s="3" t="n"/>
@@ -917,13 +944,56 @@
       <c r="K13" s="3" t="n"/>
       <c r="L13" s="3" t="n"/>
     </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Bewirtungsbeleg</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="5">
+        <f>SUMIF(C2:C6,A14,E2:E6)</f>
+        <v/>
+      </c>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="n"/>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="5">
+        <f>SUMIF(C2:C6,A15,E2:E6)</f>
+        <v/>
+      </c>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L5"/>
+  <autoFilter ref="A1:L6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>